<commit_message>
Hepatitis parent code added
</commit_message>
<xml_diff>
--- a/input/excel/Profile and ValueSet_ServiceRequest_Lab_16.01.2026/SRLabResearchs.xlsx
+++ b/input/excel/Profile and ValueSet_ServiceRequest_Lab_16.01.2026/SRLabResearchs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\behzod_axmedov\Desktop\DHP-temp02\UZCoreServiceRequest_Lab\digital-health-ig\input\excel\Profile and ValueSet_ServiceRequest_Lab_16.01.2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3BC742-4F44-4EB6-8CD9-8D7D94D56E38}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AEDDD82-D3E6-40EA-93EA-6A78716C1BA8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1370" uniqueCount="1250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1374" uniqueCount="1254">
   <si>
     <t>https://terminology.dhp.uz/fhir/core/CodeSystem/service-request-lab-research-codes-cs</t>
   </si>
@@ -3798,6 +3798,18 @@
   </si>
   <si>
     <t>lab-258</t>
+  </si>
+  <si>
+    <t>lab-P</t>
+  </si>
+  <si>
+    <t>Gepatit</t>
+  </si>
+  <si>
+    <t>Гепатит</t>
+  </si>
+  <si>
+    <t>Hepatitis</t>
   </si>
 </sst>
 </file>
@@ -3952,7 +3964,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4024,6 +4036,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -4305,7 +4322,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L275"/>
+  <dimension ref="A1:L276"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.140625" customWidth="1"/>
@@ -10522,273 +10539,288 @@
     </row>
     <row r="260" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A260" s="22" t="s">
-        <v>1234</v>
-      </c>
-      <c r="B260" s="17" t="s">
-        <v>916</v>
-      </c>
-      <c r="C260" s="18" t="s">
-        <v>917</v>
-      </c>
-      <c r="D260" s="16" t="s">
-        <v>918</v>
-      </c>
-      <c r="E260" s="17" t="s">
-        <v>919</v>
+        <v>1250</v>
+      </c>
+      <c r="B260" s="27"/>
+      <c r="C260" s="28" t="s">
+        <v>1251</v>
+      </c>
+      <c r="D260" s="29" t="s">
+        <v>1252</v>
+      </c>
+      <c r="E260" s="29" t="s">
+        <v>1253</v>
       </c>
     </row>
     <row r="261" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A261" s="22" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="B261" s="17" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="C261" s="18" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="D261" s="16" t="s">
-        <v>922</v>
+        <v>918</v>
       </c>
       <c r="E261" s="17" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
     </row>
     <row r="262" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A262" s="22" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="B262" s="17" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="C262" s="18" t="s">
-        <v>925</v>
-      </c>
-      <c r="D262" s="14" t="s">
-        <v>926</v>
+        <v>921</v>
+      </c>
+      <c r="D262" s="16" t="s">
+        <v>922</v>
       </c>
       <c r="E262" s="17" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
     </row>
     <row r="263" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A263" s="22" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="B263" s="17" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
       <c r="C263" s="18" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="D263" s="14" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
       <c r="E263" s="17" t="s">
-        <v>931</v>
+        <v>927</v>
       </c>
     </row>
     <row r="264" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A264" s="22" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="B264" s="17" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
       <c r="C264" s="18" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="D264" s="14" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
       <c r="E264" s="17" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
     </row>
     <row r="265" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A265" s="22" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="B265" s="17" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
       <c r="C265" s="18" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="D265" s="14" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
       <c r="E265" s="17" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
     </row>
     <row r="266" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A266" s="22" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="B266" s="17" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="C266" s="18" t="s">
-        <v>941</v>
+        <v>937</v>
       </c>
       <c r="D266" s="14" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
       <c r="E266" s="17" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
     </row>
     <row r="267" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A267" s="22" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="B267" s="17" t="s">
-        <v>944</v>
+        <v>940</v>
       </c>
       <c r="C267" s="18" t="s">
-        <v>945</v>
-      </c>
-      <c r="D267" s="17" t="s">
-        <v>946</v>
+        <v>941</v>
+      </c>
+      <c r="D267" s="14" t="s">
+        <v>942</v>
       </c>
       <c r="E267" s="17" t="s">
-        <v>947</v>
+        <v>943</v>
       </c>
     </row>
     <row r="268" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A268" s="22" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="B268" s="17" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
       <c r="C268" s="18" t="s">
-        <v>949</v>
-      </c>
-      <c r="D268" s="19" t="s">
-        <v>950</v>
+        <v>945</v>
+      </c>
+      <c r="D268" s="17" t="s">
+        <v>946</v>
       </c>
       <c r="E268" s="17" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
     </row>
     <row r="269" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A269" s="22" t="s">
-        <v>1243</v>
-      </c>
-      <c r="B269" s="14" t="s">
-        <v>952</v>
+        <v>1242</v>
+      </c>
+      <c r="B269" s="17" t="s">
+        <v>948</v>
       </c>
       <c r="C269" s="18" t="s">
-        <v>953</v>
-      </c>
-      <c r="D269" s="17" t="s">
-        <v>954</v>
+        <v>949</v>
+      </c>
+      <c r="D269" s="19" t="s">
+        <v>950</v>
       </c>
       <c r="E269" s="17" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
     </row>
     <row r="270" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A270" s="22" t="s">
-        <v>1244</v>
-      </c>
-      <c r="B270" s="17" t="s">
-        <v>948</v>
+        <v>1243</v>
+      </c>
+      <c r="B270" s="14" t="s">
+        <v>952</v>
       </c>
       <c r="C270" s="18" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
       <c r="D270" s="17" t="s">
-        <v>957</v>
+        <v>954</v>
       </c>
       <c r="E270" s="17" t="s">
-        <v>958</v>
+        <v>955</v>
       </c>
     </row>
     <row r="271" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A271" s="22" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="B271" s="17" t="s">
-        <v>959</v>
+        <v>948</v>
       </c>
       <c r="C271" s="18" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
       <c r="D271" s="17" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="E271" s="17" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
     </row>
     <row r="272" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A272" s="22" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="B272" s="17" t="s">
-        <v>963</v>
+        <v>959</v>
       </c>
       <c r="C272" s="18" t="s">
-        <v>964</v>
-      </c>
-      <c r="D272" s="15" t="s">
-        <v>965</v>
-      </c>
-      <c r="E272" s="20" t="s">
-        <v>966</v>
+        <v>960</v>
+      </c>
+      <c r="D272" s="17" t="s">
+        <v>961</v>
+      </c>
+      <c r="E272" s="17" t="s">
+        <v>962</v>
       </c>
     </row>
     <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="22" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="B273" s="17" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="C273" s="18" t="s">
-        <v>968</v>
-      </c>
-      <c r="D273" s="17" t="s">
-        <v>969</v>
-      </c>
-      <c r="E273" s="17" t="s">
-        <v>970</v>
+        <v>964</v>
+      </c>
+      <c r="D273" s="15" t="s">
+        <v>965</v>
+      </c>
+      <c r="E273" s="20" t="s">
+        <v>966</v>
       </c>
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="22" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="B274" s="17" t="s">
-        <v>971</v>
+        <v>967</v>
       </c>
       <c r="C274" s="18" t="s">
-        <v>972</v>
+        <v>968</v>
       </c>
       <c r="D274" s="17" t="s">
-        <v>973</v>
-      </c>
-      <c r="E274" s="21" t="s">
-        <v>974</v>
+        <v>969</v>
+      </c>
+      <c r="E274" s="17" t="s">
+        <v>970</v>
       </c>
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="22" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B275" s="17" t="s">
+        <v>971</v>
+      </c>
+      <c r="C275" s="18" t="s">
+        <v>972</v>
+      </c>
+      <c r="D275" s="17" t="s">
+        <v>973</v>
+      </c>
+      <c r="E275" s="21" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A276" s="22" t="s">
         <v>1249</v>
       </c>
-      <c r="B275" s="17" t="s">
+      <c r="B276" s="17" t="s">
         <v>975</v>
       </c>
-      <c r="C275" s="18" t="s">
+      <c r="C276" s="18" t="s">
         <v>976</v>
       </c>
-      <c r="D275" s="17" t="s">
+      <c r="D276" s="17" t="s">
         <v>977</v>
       </c>
-      <c r="E275" s="17" t="s">
+      <c r="E276" s="17" t="s">
         <v>978</v>
       </c>
     </row>

</xml_diff>